<commit_message>
Echo waveform & spectrum
</commit_message>
<xml_diff>
--- a/planning.xlsx
+++ b/planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8564a8c591b3536d/Documenten/Uni/Thesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="8_{E3DC4D32-73A5-476F-9434-1C62C3491628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E335B255-E423-4C6B-921C-DD9003E1C4AA}"/>
+  <xr:revisionPtr revIDLastSave="280" documentId="8_{E3DC4D32-73A5-476F-9434-1C62C3491628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37A081AD-B0A9-412B-9144-C7AB51AB3ACB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="52">
   <si>
     <t>Project start:</t>
   </si>
@@ -73,33 +73,6 @@
   </si>
   <si>
     <t xml:space="preserve">Do not delete this row. This row is hidden to preserve a formula that is used to highlight the current day within the project schedule. </t>
-  </si>
-  <si>
-    <t>Define scope</t>
-  </si>
-  <si>
-    <t>Identify risks</t>
-  </si>
-  <si>
-    <t>Monitor progress</t>
-  </si>
-  <si>
-    <t>Provide updates</t>
-  </si>
-  <si>
-    <t>Testing and validation</t>
-  </si>
-  <si>
-    <t>Track expenses</t>
-  </si>
-  <si>
-    <t>Evaluate progress</t>
-  </si>
-  <si>
-    <t>Address risks</t>
-  </si>
-  <si>
-    <t>Gather feedback</t>
   </si>
   <si>
     <t>About This Template</t>
@@ -173,12 +146,6 @@
     <t>Prelimenairy model</t>
   </si>
   <si>
-    <t>Literature study (SOTA)</t>
-  </si>
-  <si>
-    <t>Identify variables</t>
-  </si>
-  <si>
     <t>Jacobs Brent</t>
   </si>
   <si>
@@ -203,9 +170,6 @@
     <t>Planning &amp; Lit review deadline</t>
   </si>
   <si>
-    <t>First budget estimation</t>
-  </si>
-  <si>
     <t>Non-technical</t>
   </si>
   <si>
@@ -216,6 +180,36 @@
   </si>
   <si>
     <t>Final Text</t>
+  </si>
+  <si>
+    <t>SoTA</t>
+  </si>
+  <si>
+    <t>Literature study</t>
+  </si>
+  <si>
+    <t>Assembly</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>choose µprocessor</t>
+  </si>
+  <si>
+    <t>Write code</t>
+  </si>
+  <si>
+    <t>Spec 2 Spec</t>
+  </si>
+  <si>
+    <t>First FEB budget</t>
+  </si>
+  <si>
+    <t>Final FEB budget</t>
+  </si>
+  <si>
+    <t>Build simulator</t>
   </si>
 </sst>
 </file>
@@ -1065,6 +1059,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1085,19 +1092,6 @@
     <xf numFmtId="167" fontId="15" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="14">
     <cellStyle name="Bad" xfId="13" builtinId="27"/>
@@ -1717,64 +1711,64 @@
     <row r="1" spans="1:63" ht="90" customHeight="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A1" s="72"/>
       <c r="B1" s="64" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C1" s="14"/>
       <c r="D1" s="15"/>
       <c r="E1" s="16"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="106" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="102"/>
-      <c r="J1" s="102"/>
-      <c r="K1" s="102"/>
-      <c r="L1" s="102"/>
-      <c r="M1" s="102"/>
-      <c r="N1" s="102"/>
+      <c r="I1" s="107"/>
+      <c r="J1" s="107"/>
+      <c r="K1" s="107"/>
+      <c r="L1" s="107"/>
+      <c r="M1" s="107"/>
+      <c r="N1" s="107"/>
       <c r="O1" s="19"/>
-      <c r="P1" s="100">
+      <c r="P1" s="105">
         <v>46286</v>
       </c>
-      <c r="Q1" s="99"/>
-      <c r="R1" s="99"/>
-      <c r="S1" s="99"/>
-      <c r="T1" s="99"/>
-      <c r="U1" s="99"/>
-      <c r="V1" s="99"/>
-      <c r="W1" s="99"/>
-      <c r="X1" s="99"/>
-      <c r="Y1" s="99"/>
+      <c r="Q1" s="104"/>
+      <c r="R1" s="104"/>
+      <c r="S1" s="104"/>
+      <c r="T1" s="104"/>
+      <c r="U1" s="104"/>
+      <c r="V1" s="104"/>
+      <c r="W1" s="104"/>
+      <c r="X1" s="104"/>
+      <c r="Y1" s="104"/>
     </row>
     <row r="2" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B2" s="63" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="18"/>
       <c r="E2" s="17"/>
-      <c r="H2" s="101" t="s">
+      <c r="H2" s="106" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="102"/>
-      <c r="J2" s="102"/>
-      <c r="K2" s="102"/>
-      <c r="L2" s="102"/>
-      <c r="M2" s="102"/>
-      <c r="N2" s="102"/>
+      <c r="I2" s="107"/>
+      <c r="J2" s="107"/>
+      <c r="K2" s="107"/>
+      <c r="L2" s="107"/>
+      <c r="M2" s="107"/>
+      <c r="N2" s="107"/>
       <c r="O2" s="19"/>
-      <c r="P2" s="98">
-        <v>3</v>
-      </c>
-      <c r="Q2" s="99"/>
-      <c r="R2" s="99"/>
-      <c r="S2" s="99"/>
-      <c r="T2" s="99"/>
-      <c r="U2" s="99"/>
-      <c r="V2" s="99"/>
-      <c r="W2" s="99"/>
-      <c r="X2" s="99"/>
-      <c r="Y2" s="99"/>
+      <c r="P2" s="103">
+        <v>4</v>
+      </c>
+      <c r="Q2" s="104"/>
+      <c r="R2" s="104"/>
+      <c r="S2" s="104"/>
+      <c r="T2" s="104"/>
+      <c r="U2" s="104"/>
+      <c r="V2" s="104"/>
+      <c r="W2" s="104"/>
+      <c r="X2" s="104"/>
+      <c r="Y2" s="104"/>
     </row>
     <row r="3" spans="1:63" s="20" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11"/>
@@ -1788,332 +1782,332 @@
       <c r="A4" s="72"/>
       <c r="B4" s="97"/>
       <c r="D4" s="23"/>
-      <c r="H4" s="105">
+      <c r="H4" s="110">
         <f>H5</f>
-        <v>46300</v>
-      </c>
-      <c r="I4" s="103"/>
-      <c r="J4" s="103"/>
-      <c r="K4" s="103"/>
-      <c r="L4" s="103"/>
-      <c r="M4" s="103"/>
-      <c r="N4" s="103"/>
-      <c r="O4" s="103">
+        <v>46307</v>
+      </c>
+      <c r="I4" s="108"/>
+      <c r="J4" s="108"/>
+      <c r="K4" s="108"/>
+      <c r="L4" s="108"/>
+      <c r="M4" s="108"/>
+      <c r="N4" s="108"/>
+      <c r="O4" s="108">
         <f>O5</f>
-        <v>46307</v>
-      </c>
-      <c r="P4" s="103"/>
-      <c r="Q4" s="103"/>
-      <c r="R4" s="103"/>
-      <c r="S4" s="103"/>
-      <c r="T4" s="103"/>
-      <c r="U4" s="103"/>
-      <c r="V4" s="103">
+        <v>46314</v>
+      </c>
+      <c r="P4" s="108"/>
+      <c r="Q4" s="108"/>
+      <c r="R4" s="108"/>
+      <c r="S4" s="108"/>
+      <c r="T4" s="108"/>
+      <c r="U4" s="108"/>
+      <c r="V4" s="108">
         <f>V5</f>
-        <v>46314</v>
-      </c>
-      <c r="W4" s="103"/>
-      <c r="X4" s="103"/>
-      <c r="Y4" s="103"/>
-      <c r="Z4" s="103"/>
-      <c r="AA4" s="103"/>
-      <c r="AB4" s="103"/>
-      <c r="AC4" s="103">
+        <v>46321</v>
+      </c>
+      <c r="W4" s="108"/>
+      <c r="X4" s="108"/>
+      <c r="Y4" s="108"/>
+      <c r="Z4" s="108"/>
+      <c r="AA4" s="108"/>
+      <c r="AB4" s="108"/>
+      <c r="AC4" s="108">
         <f>AC5</f>
-        <v>46321</v>
-      </c>
-      <c r="AD4" s="103"/>
-      <c r="AE4" s="103"/>
-      <c r="AF4" s="103"/>
-      <c r="AG4" s="103"/>
-      <c r="AH4" s="103"/>
-      <c r="AI4" s="103"/>
-      <c r="AJ4" s="103">
+        <v>46328</v>
+      </c>
+      <c r="AD4" s="108"/>
+      <c r="AE4" s="108"/>
+      <c r="AF4" s="108"/>
+      <c r="AG4" s="108"/>
+      <c r="AH4" s="108"/>
+      <c r="AI4" s="108"/>
+      <c r="AJ4" s="108">
         <f>AJ5</f>
-        <v>46328</v>
-      </c>
-      <c r="AK4" s="103"/>
-      <c r="AL4" s="103"/>
-      <c r="AM4" s="103"/>
-      <c r="AN4" s="103"/>
-      <c r="AO4" s="103"/>
-      <c r="AP4" s="103"/>
-      <c r="AQ4" s="103">
+        <v>46335</v>
+      </c>
+      <c r="AK4" s="108"/>
+      <c r="AL4" s="108"/>
+      <c r="AM4" s="108"/>
+      <c r="AN4" s="108"/>
+      <c r="AO4" s="108"/>
+      <c r="AP4" s="108"/>
+      <c r="AQ4" s="108">
         <f>AQ5</f>
-        <v>46335</v>
-      </c>
-      <c r="AR4" s="103"/>
-      <c r="AS4" s="103"/>
-      <c r="AT4" s="103"/>
-      <c r="AU4" s="103"/>
-      <c r="AV4" s="103"/>
-      <c r="AW4" s="103"/>
-      <c r="AX4" s="103">
+        <v>46342</v>
+      </c>
+      <c r="AR4" s="108"/>
+      <c r="AS4" s="108"/>
+      <c r="AT4" s="108"/>
+      <c r="AU4" s="108"/>
+      <c r="AV4" s="108"/>
+      <c r="AW4" s="108"/>
+      <c r="AX4" s="108">
         <f>AX5</f>
-        <v>46342</v>
-      </c>
-      <c r="AY4" s="103"/>
-      <c r="AZ4" s="103"/>
-      <c r="BA4" s="103"/>
-      <c r="BB4" s="103"/>
-      <c r="BC4" s="103"/>
-      <c r="BD4" s="103"/>
-      <c r="BE4" s="103">
+        <v>46349</v>
+      </c>
+      <c r="AY4" s="108"/>
+      <c r="AZ4" s="108"/>
+      <c r="BA4" s="108"/>
+      <c r="BB4" s="108"/>
+      <c r="BC4" s="108"/>
+      <c r="BD4" s="108"/>
+      <c r="BE4" s="108">
         <f>BE5</f>
-        <v>46349</v>
-      </c>
-      <c r="BF4" s="103"/>
-      <c r="BG4" s="103"/>
-      <c r="BH4" s="103"/>
-      <c r="BI4" s="103"/>
-      <c r="BJ4" s="103"/>
-      <c r="BK4" s="104"/>
+        <v>46356</v>
+      </c>
+      <c r="BF4" s="108"/>
+      <c r="BG4" s="108"/>
+      <c r="BH4" s="108"/>
+      <c r="BI4" s="108"/>
+      <c r="BJ4" s="108"/>
+      <c r="BK4" s="109"/>
     </row>
     <row r="5" spans="1:63" s="20" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="106"/>
-      <c r="B5" s="107" t="s">
+      <c r="A5" s="98"/>
+      <c r="B5" s="99" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="109" t="s">
+      <c r="C5" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="109" t="s">
+      <c r="D5" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="109" t="s">
+      <c r="E5" s="101" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="24">
         <f>Project_Start-WEEKDAY(Project_Start,1)+2+7*(Display_Week-1)</f>
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="I5" s="24">
         <f>H5+1</f>
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="J5" s="24">
         <f t="shared" ref="J5:AW5" si="0">I5+1</f>
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="K5" s="24">
         <f t="shared" si="0"/>
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="L5" s="24">
         <f t="shared" si="0"/>
-        <v>46304</v>
+        <v>46311</v>
       </c>
       <c r="M5" s="24">
         <f t="shared" si="0"/>
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="N5" s="25">
         <f t="shared" si="0"/>
-        <v>46306</v>
+        <v>46313</v>
       </c>
       <c r="O5" s="26">
         <f>N5+1</f>
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="P5" s="24">
         <f>O5+1</f>
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="Q5" s="24">
         <f t="shared" si="0"/>
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="R5" s="24">
         <f t="shared" si="0"/>
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="S5" s="24">
         <f t="shared" si="0"/>
-        <v>46311</v>
+        <v>46318</v>
       </c>
       <c r="T5" s="24">
         <f t="shared" si="0"/>
-        <v>46312</v>
+        <v>46319</v>
       </c>
       <c r="U5" s="25">
         <f t="shared" si="0"/>
-        <v>46313</v>
+        <v>46320</v>
       </c>
       <c r="V5" s="26">
         <f>U5+1</f>
-        <v>46314</v>
+        <v>46321</v>
       </c>
       <c r="W5" s="24">
         <f>V5+1</f>
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="X5" s="24">
         <f t="shared" si="0"/>
-        <v>46316</v>
+        <v>46323</v>
       </c>
       <c r="Y5" s="24">
         <f t="shared" si="0"/>
-        <v>46317</v>
+        <v>46324</v>
       </c>
       <c r="Z5" s="24">
         <f t="shared" si="0"/>
-        <v>46318</v>
+        <v>46325</v>
       </c>
       <c r="AA5" s="24">
         <f t="shared" si="0"/>
-        <v>46319</v>
+        <v>46326</v>
       </c>
       <c r="AB5" s="25">
         <f t="shared" si="0"/>
-        <v>46320</v>
+        <v>46327</v>
       </c>
       <c r="AC5" s="26">
         <f>AB5+1</f>
-        <v>46321</v>
+        <v>46328</v>
       </c>
       <c r="AD5" s="24">
         <f>AC5+1</f>
-        <v>46322</v>
+        <v>46329</v>
       </c>
       <c r="AE5" s="24">
         <f t="shared" si="0"/>
-        <v>46323</v>
+        <v>46330</v>
       </c>
       <c r="AF5" s="24">
         <f t="shared" si="0"/>
-        <v>46324</v>
+        <v>46331</v>
       </c>
       <c r="AG5" s="24">
         <f t="shared" si="0"/>
-        <v>46325</v>
+        <v>46332</v>
       </c>
       <c r="AH5" s="24">
         <f t="shared" si="0"/>
-        <v>46326</v>
+        <v>46333</v>
       </c>
       <c r="AI5" s="25">
         <f t="shared" si="0"/>
-        <v>46327</v>
+        <v>46334</v>
       </c>
       <c r="AJ5" s="26">
         <f>AI5+1</f>
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="AK5" s="24">
         <f>AJ5+1</f>
-        <v>46329</v>
+        <v>46336</v>
       </c>
       <c r="AL5" s="24">
         <f t="shared" si="0"/>
-        <v>46330</v>
+        <v>46337</v>
       </c>
       <c r="AM5" s="24">
         <f t="shared" si="0"/>
-        <v>46331</v>
+        <v>46338</v>
       </c>
       <c r="AN5" s="24">
         <f t="shared" si="0"/>
-        <v>46332</v>
+        <v>46339</v>
       </c>
       <c r="AO5" s="24">
         <f t="shared" si="0"/>
-        <v>46333</v>
+        <v>46340</v>
       </c>
       <c r="AP5" s="25">
         <f t="shared" si="0"/>
-        <v>46334</v>
+        <v>46341</v>
       </c>
       <c r="AQ5" s="26">
         <f>AP5+1</f>
-        <v>46335</v>
+        <v>46342</v>
       </c>
       <c r="AR5" s="24">
         <f>AQ5+1</f>
-        <v>46336</v>
+        <v>46343</v>
       </c>
       <c r="AS5" s="24">
         <f t="shared" si="0"/>
-        <v>46337</v>
+        <v>46344</v>
       </c>
       <c r="AT5" s="24">
         <f t="shared" si="0"/>
-        <v>46338</v>
+        <v>46345</v>
       </c>
       <c r="AU5" s="24">
         <f t="shared" si="0"/>
-        <v>46339</v>
+        <v>46346</v>
       </c>
       <c r="AV5" s="24">
         <f t="shared" si="0"/>
-        <v>46340</v>
+        <v>46347</v>
       </c>
       <c r="AW5" s="25">
         <f t="shared" si="0"/>
-        <v>46341</v>
+        <v>46348</v>
       </c>
       <c r="AX5" s="26">
         <f>AW5+1</f>
-        <v>46342</v>
+        <v>46349</v>
       </c>
       <c r="AY5" s="24">
         <f>AX5+1</f>
-        <v>46343</v>
+        <v>46350</v>
       </c>
       <c r="AZ5" s="24">
         <f t="shared" ref="AZ5:BD5" si="1">AY5+1</f>
-        <v>46344</v>
+        <v>46351</v>
       </c>
       <c r="BA5" s="24">
         <f t="shared" si="1"/>
-        <v>46345</v>
+        <v>46352</v>
       </c>
       <c r="BB5" s="24">
         <f t="shared" si="1"/>
-        <v>46346</v>
+        <v>46353</v>
       </c>
       <c r="BC5" s="24">
         <f t="shared" si="1"/>
-        <v>46347</v>
+        <v>46354</v>
       </c>
       <c r="BD5" s="25">
         <f t="shared" si="1"/>
-        <v>46348</v>
+        <v>46355</v>
       </c>
       <c r="BE5" s="26">
         <f>BD5+1</f>
-        <v>46349</v>
+        <v>46356</v>
       </c>
       <c r="BF5" s="24">
         <f>BE5+1</f>
-        <v>46350</v>
+        <v>46357</v>
       </c>
       <c r="BG5" s="24">
         <f t="shared" ref="BG5:BK5" si="2">BF5+1</f>
-        <v>46351</v>
+        <v>46358</v>
       </c>
       <c r="BH5" s="24">
         <f t="shared" si="2"/>
-        <v>46352</v>
+        <v>46359</v>
       </c>
       <c r="BI5" s="24">
         <f t="shared" si="2"/>
-        <v>46353</v>
+        <v>46360</v>
       </c>
       <c r="BJ5" s="24">
         <f t="shared" si="2"/>
-        <v>46354</v>
+        <v>46361</v>
       </c>
       <c r="BK5" s="24">
         <f t="shared" si="2"/>
-        <v>46355</v>
+        <v>46362</v>
       </c>
     </row>
     <row r="6" spans="1:63" s="20" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="106"/>
-      <c r="B6" s="108"/>
-      <c r="C6" s="110"/>
-      <c r="D6" s="110"/>
-      <c r="E6" s="110"/>
+      <c r="A6" s="98"/>
+      <c r="B6" s="100"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
       <c r="H6" s="27" t="str">
         <f t="shared" ref="H6:AM6" si="3">LEFT(TEXT(H5,"ddd"),1)</f>
         <v>M</v>
@@ -2411,7 +2405,7 @@
     <row r="8" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="72"/>
       <c r="B8" s="32" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="C8" s="33"/>
       <c r="D8" s="34"/>
@@ -2481,7 +2475,7 @@
     <row r="9" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="72"/>
       <c r="B9" s="38" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="C9" s="39">
         <v>1</v>
@@ -2558,10 +2552,10 @@
     <row r="10" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="72"/>
       <c r="B10" s="41" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C10" s="42">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="D10" s="81">
         <v>46286</v>
@@ -2634,7 +2628,7 @@
     <row r="11" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="72"/>
       <c r="B11" s="41" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C11" s="42">
         <v>0</v>
@@ -2707,16 +2701,16 @@
     <row r="12" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="72"/>
       <c r="B12" s="41" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C12" s="42">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D12" s="81">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="E12" s="81">
-        <v>46327</v>
+        <v>46309</v>
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="4"/>
@@ -2777,101 +2771,95 @@
       <c r="BJ12" s="40"/>
       <c r="BK12" s="40"/>
     </row>
-    <row r="13" spans="1:63" s="89" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="82"/>
-      <c r="B13" s="83" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="84">
-        <v>0.1</v>
-      </c>
-      <c r="D13" s="85">
+    <row r="13" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="72"/>
+      <c r="B13" s="41" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="42">
+        <v>0.4</v>
+      </c>
+      <c r="D13" s="81">
+        <v>46309</v>
+      </c>
+      <c r="E13" s="81">
         <v>46327</v>
       </c>
-      <c r="E13" s="85">
+      <c r="F13" s="13"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="40"/>
+      <c r="K13" s="40"/>
+      <c r="L13" s="40"/>
+      <c r="M13" s="40"/>
+      <c r="N13" s="40"/>
+      <c r="O13" s="40"/>
+      <c r="P13" s="40"/>
+      <c r="Q13" s="40"/>
+      <c r="R13" s="40"/>
+      <c r="S13" s="40"/>
+      <c r="T13" s="43"/>
+      <c r="U13" s="43"/>
+      <c r="V13" s="40"/>
+      <c r="W13" s="40"/>
+      <c r="X13" s="40"/>
+      <c r="Y13" s="40"/>
+      <c r="Z13" s="40"/>
+      <c r="AA13" s="40"/>
+      <c r="AB13" s="40"/>
+      <c r="AC13" s="40"/>
+      <c r="AD13" s="40"/>
+      <c r="AE13" s="40"/>
+      <c r="AF13" s="40"/>
+      <c r="AG13" s="40"/>
+      <c r="AH13" s="40"/>
+      <c r="AI13" s="40"/>
+      <c r="AJ13" s="40"/>
+      <c r="AK13" s="40"/>
+      <c r="AL13" s="40"/>
+      <c r="AM13" s="40"/>
+      <c r="AN13" s="40"/>
+      <c r="AO13" s="40"/>
+      <c r="AP13" s="40"/>
+      <c r="AQ13" s="40"/>
+      <c r="AR13" s="40"/>
+      <c r="AS13" s="40"/>
+      <c r="AT13" s="40"/>
+      <c r="AU13" s="40"/>
+      <c r="AV13" s="40"/>
+      <c r="AW13" s="40"/>
+      <c r="AX13" s="40"/>
+      <c r="AY13" s="40"/>
+      <c r="AZ13" s="40"/>
+      <c r="BA13" s="40"/>
+      <c r="BB13" s="40"/>
+      <c r="BC13" s="40"/>
+      <c r="BD13" s="40"/>
+      <c r="BE13" s="40"/>
+      <c r="BF13" s="40"/>
+      <c r="BG13" s="40"/>
+      <c r="BH13" s="40"/>
+      <c r="BI13" s="40"/>
+      <c r="BJ13" s="40"/>
+      <c r="BK13" s="40"/>
+    </row>
+    <row r="14" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="72"/>
+      <c r="B14" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="42">
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="81">
+        <v>46300</v>
+      </c>
+      <c r="E14" s="81">
         <v>46327</v>
       </c>
-      <c r="F13" s="86"/>
-      <c r="G13" s="87">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-      <c r="H13" s="88"/>
-      <c r="I13" s="88"/>
-      <c r="J13" s="88"/>
-      <c r="K13" s="88"/>
-      <c r="L13" s="88"/>
-      <c r="M13" s="88"/>
-      <c r="N13" s="88"/>
-      <c r="O13" s="88"/>
-      <c r="P13" s="88"/>
-      <c r="Q13" s="88"/>
-      <c r="R13" s="88"/>
-      <c r="S13" s="88"/>
-      <c r="T13" s="88"/>
-      <c r="U13" s="88"/>
-      <c r="V13" s="88"/>
-      <c r="W13" s="88"/>
-      <c r="X13" s="88"/>
-      <c r="Y13" s="88"/>
-      <c r="Z13" s="88"/>
-      <c r="AA13" s="88"/>
-      <c r="AB13" s="88"/>
-      <c r="AC13" s="88"/>
-      <c r="AD13" s="88"/>
-      <c r="AE13" s="88"/>
-      <c r="AF13" s="88"/>
-      <c r="AG13" s="88"/>
-      <c r="AH13" s="88"/>
-      <c r="AI13" s="88"/>
-      <c r="AJ13" s="88"/>
-      <c r="AK13" s="88"/>
-      <c r="AL13" s="88"/>
-      <c r="AM13" s="88"/>
-      <c r="AN13" s="88"/>
-      <c r="AO13" s="88"/>
-      <c r="AP13" s="88"/>
-      <c r="AQ13" s="88"/>
-      <c r="AR13" s="88"/>
-      <c r="AS13" s="88"/>
-      <c r="AT13" s="88"/>
-      <c r="AU13" s="88"/>
-      <c r="AV13" s="88"/>
-      <c r="AW13" s="88"/>
-      <c r="AX13" s="88"/>
-      <c r="AY13" s="88"/>
-      <c r="AZ13" s="88"/>
-      <c r="BA13" s="88"/>
-      <c r="BB13" s="88"/>
-      <c r="BC13" s="88"/>
-      <c r="BD13" s="88"/>
-      <c r="BE13" s="88"/>
-      <c r="BF13" s="88"/>
-      <c r="BG13" s="88"/>
-      <c r="BH13" s="88"/>
-      <c r="BI13" s="88"/>
-      <c r="BJ13" s="88"/>
-      <c r="BK13" s="88"/>
-    </row>
-    <row r="14" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="42">
-        <v>0</v>
-      </c>
-      <c r="D14" s="81">
-        <v>46327</v>
-      </c>
-      <c r="E14" s="81">
-        <v>46370</v>
-      </c>
       <c r="F14" s="13"/>
-      <c r="G14" s="4">
-        <f t="shared" si="5"/>
-        <v>44</v>
-      </c>
+      <c r="G14" s="4"/>
       <c r="H14" s="40"/>
       <c r="I14" s="40"/>
       <c r="J14" s="40"/>
@@ -2884,11 +2872,11 @@
       <c r="Q14" s="40"/>
       <c r="R14" s="40"/>
       <c r="S14" s="40"/>
-      <c r="T14" s="40"/>
-      <c r="U14" s="40"/>
+      <c r="T14" s="43"/>
+      <c r="U14" s="43"/>
       <c r="V14" s="40"/>
       <c r="W14" s="40"/>
-      <c r="X14" s="43"/>
+      <c r="X14" s="40"/>
       <c r="Y14" s="40"/>
       <c r="Z14" s="40"/>
       <c r="AA14" s="40"/>
@@ -2929,95 +2917,101 @@
       <c r="BJ14" s="40"/>
       <c r="BK14" s="40"/>
     </row>
-    <row r="15" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="42">
-        <v>0</v>
-      </c>
-      <c r="D15" s="81">
+    <row r="15" spans="1:63" s="89" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="82"/>
+      <c r="B15" s="83" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="84">
+        <v>0.1</v>
+      </c>
+      <c r="D15" s="85">
+        <v>46324</v>
+      </c>
+      <c r="E15" s="85">
         <v>46327</v>
       </c>
-      <c r="E15" s="81">
-        <v>46334</v>
-      </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="40"/>
-      <c r="K15" s="40"/>
-      <c r="L15" s="40"/>
-      <c r="M15" s="40"/>
-      <c r="N15" s="40"/>
-      <c r="O15" s="40"/>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="40"/>
-      <c r="R15" s="40"/>
-      <c r="S15" s="40"/>
-      <c r="T15" s="40"/>
-      <c r="U15" s="40"/>
-      <c r="V15" s="40"/>
-      <c r="W15" s="40"/>
-      <c r="X15" s="43"/>
-      <c r="Y15" s="40"/>
-      <c r="Z15" s="40"/>
-      <c r="AA15" s="40"/>
-      <c r="AB15" s="40"/>
-      <c r="AC15" s="40"/>
-      <c r="AD15" s="40"/>
-      <c r="AE15" s="40"/>
-      <c r="AF15" s="40"/>
-      <c r="AG15" s="40"/>
-      <c r="AH15" s="40"/>
-      <c r="AI15" s="40"/>
-      <c r="AJ15" s="40"/>
-      <c r="AK15" s="40"/>
-      <c r="AL15" s="40"/>
-      <c r="AM15" s="40"/>
-      <c r="AN15" s="40"/>
-      <c r="AO15" s="40"/>
-      <c r="AP15" s="40"/>
-      <c r="AQ15" s="40"/>
-      <c r="AR15" s="40"/>
-      <c r="AS15" s="40"/>
-      <c r="AT15" s="40"/>
-      <c r="AU15" s="40"/>
-      <c r="AV15" s="40"/>
-      <c r="AW15" s="40"/>
-      <c r="AX15" s="40"/>
-      <c r="AY15" s="40"/>
-      <c r="AZ15" s="40"/>
-      <c r="BA15" s="40"/>
-      <c r="BB15" s="40"/>
-      <c r="BC15" s="40"/>
-      <c r="BD15" s="40"/>
-      <c r="BE15" s="40"/>
-      <c r="BF15" s="40"/>
-      <c r="BG15" s="40"/>
-      <c r="BH15" s="40"/>
-      <c r="BI15" s="40"/>
-      <c r="BJ15" s="40"/>
-      <c r="BK15" s="40"/>
+      <c r="F15" s="86"/>
+      <c r="G15" s="87">
+        <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="H15" s="88"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="88"/>
+      <c r="K15" s="88"/>
+      <c r="L15" s="88"/>
+      <c r="M15" s="88"/>
+      <c r="N15" s="88"/>
+      <c r="O15" s="88"/>
+      <c r="P15" s="88"/>
+      <c r="Q15" s="88"/>
+      <c r="R15" s="88"/>
+      <c r="S15" s="88"/>
+      <c r="T15" s="88"/>
+      <c r="U15" s="88"/>
+      <c r="V15" s="88"/>
+      <c r="W15" s="88"/>
+      <c r="X15" s="88"/>
+      <c r="Y15" s="88"/>
+      <c r="Z15" s="88"/>
+      <c r="AA15" s="88"/>
+      <c r="AB15" s="88"/>
+      <c r="AC15" s="88"/>
+      <c r="AD15" s="88"/>
+      <c r="AE15" s="88"/>
+      <c r="AF15" s="88"/>
+      <c r="AG15" s="88"/>
+      <c r="AH15" s="88"/>
+      <c r="AI15" s="88"/>
+      <c r="AJ15" s="88"/>
+      <c r="AK15" s="88"/>
+      <c r="AL15" s="88"/>
+      <c r="AM15" s="88"/>
+      <c r="AN15" s="88"/>
+      <c r="AO15" s="88"/>
+      <c r="AP15" s="88"/>
+      <c r="AQ15" s="88"/>
+      <c r="AR15" s="88"/>
+      <c r="AS15" s="88"/>
+      <c r="AT15" s="88"/>
+      <c r="AU15" s="88"/>
+      <c r="AV15" s="88"/>
+      <c r="AW15" s="88"/>
+      <c r="AX15" s="88"/>
+      <c r="AY15" s="88"/>
+      <c r="AZ15" s="88"/>
+      <c r="BA15" s="88"/>
+      <c r="BB15" s="88"/>
+      <c r="BC15" s="88"/>
+      <c r="BD15" s="88"/>
+      <c r="BE15" s="88"/>
+      <c r="BF15" s="88"/>
+      <c r="BG15" s="88"/>
+      <c r="BH15" s="88"/>
+      <c r="BI15" s="88"/>
+      <c r="BJ15" s="88"/>
+      <c r="BK15" s="88"/>
     </row>
     <row r="16" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
       <c r="B16" s="41" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C16" s="42">
         <v>0</v>
       </c>
       <c r="D16" s="81">
-        <v>46340</v>
+        <v>46327</v>
       </c>
       <c r="E16" s="81">
-        <v>46348</v>
+        <v>46370</v>
       </c>
       <c r="F16" s="13"/>
-      <c r="G16" s="4"/>
+      <c r="G16" s="4">
+        <f t="shared" si="5"/>
+        <v>44</v>
+      </c>
       <c r="H16" s="40"/>
       <c r="I16" s="40"/>
       <c r="J16" s="40"/>
@@ -3078,16 +3072,16 @@
     <row r="17" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
       <c r="B17" s="41" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="C17" s="42">
         <v>0</v>
       </c>
       <c r="D17" s="81">
-        <v>46348</v>
+        <v>46327</v>
       </c>
       <c r="E17" s="81">
-        <v>46355</v>
+        <v>46334</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="4"/>
@@ -3148,98 +3142,95 @@
       <c r="BJ17" s="40"/>
       <c r="BK17" s="40"/>
     </row>
-    <row r="18" spans="1:63" s="89" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="82"/>
-      <c r="B18" s="83" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="84">
+    <row r="18" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11"/>
+      <c r="B18" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="42">
         <v>0</v>
       </c>
-      <c r="D18" s="85">
-        <v>46374</v>
-      </c>
-      <c r="E18" s="85">
-        <v>46374</v>
-      </c>
-      <c r="F18" s="86"/>
-      <c r="G18" s="87"/>
-      <c r="H18" s="88"/>
-      <c r="I18" s="88"/>
-      <c r="J18" s="88"/>
-      <c r="K18" s="88"/>
-      <c r="L18" s="88"/>
-      <c r="M18" s="88"/>
-      <c r="N18" s="88"/>
-      <c r="O18" s="88"/>
-      <c r="P18" s="88"/>
-      <c r="Q18" s="88"/>
-      <c r="R18" s="88"/>
-      <c r="S18" s="88"/>
-      <c r="T18" s="88"/>
-      <c r="U18" s="88"/>
-      <c r="V18" s="88"/>
-      <c r="W18" s="88"/>
-      <c r="X18" s="90"/>
-      <c r="Y18" s="88"/>
-      <c r="Z18" s="88"/>
-      <c r="AA18" s="88"/>
-      <c r="AB18" s="88"/>
-      <c r="AC18" s="88"/>
-      <c r="AD18" s="88"/>
-      <c r="AE18" s="88"/>
-      <c r="AF18" s="88"/>
-      <c r="AG18" s="88"/>
-      <c r="AH18" s="88"/>
-      <c r="AI18" s="88"/>
-      <c r="AJ18" s="88"/>
-      <c r="AK18" s="88"/>
-      <c r="AL18" s="88"/>
-      <c r="AM18" s="88"/>
-      <c r="AN18" s="88"/>
-      <c r="AO18" s="88"/>
-      <c r="AP18" s="88"/>
-      <c r="AQ18" s="88"/>
-      <c r="AR18" s="88"/>
-      <c r="AS18" s="88"/>
-      <c r="AT18" s="88"/>
-      <c r="AU18" s="88"/>
-      <c r="AV18" s="88"/>
-      <c r="AW18" s="88"/>
-      <c r="AX18" s="88"/>
-      <c r="AY18" s="88"/>
-      <c r="AZ18" s="88"/>
-      <c r="BA18" s="88"/>
-      <c r="BB18" s="88"/>
-      <c r="BC18" s="88"/>
-      <c r="BD18" s="88"/>
-      <c r="BE18" s="88"/>
-      <c r="BF18" s="88"/>
-      <c r="BG18" s="88"/>
-      <c r="BH18" s="88"/>
-      <c r="BI18" s="88"/>
-      <c r="BJ18" s="88"/>
-      <c r="BK18" s="88"/>
+      <c r="D18" s="81">
+        <v>46340</v>
+      </c>
+      <c r="E18" s="81">
+        <v>46348</v>
+      </c>
+      <c r="F18" s="13"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="40"/>
+      <c r="N18" s="40"/>
+      <c r="O18" s="40"/>
+      <c r="P18" s="40"/>
+      <c r="Q18" s="40"/>
+      <c r="R18" s="40"/>
+      <c r="S18" s="40"/>
+      <c r="T18" s="40"/>
+      <c r="U18" s="40"/>
+      <c r="V18" s="40"/>
+      <c r="W18" s="40"/>
+      <c r="X18" s="43"/>
+      <c r="Y18" s="40"/>
+      <c r="Z18" s="40"/>
+      <c r="AA18" s="40"/>
+      <c r="AB18" s="40"/>
+      <c r="AC18" s="40"/>
+      <c r="AD18" s="40"/>
+      <c r="AE18" s="40"/>
+      <c r="AF18" s="40"/>
+      <c r="AG18" s="40"/>
+      <c r="AH18" s="40"/>
+      <c r="AI18" s="40"/>
+      <c r="AJ18" s="40"/>
+      <c r="AK18" s="40"/>
+      <c r="AL18" s="40"/>
+      <c r="AM18" s="40"/>
+      <c r="AN18" s="40"/>
+      <c r="AO18" s="40"/>
+      <c r="AP18" s="40"/>
+      <c r="AQ18" s="40"/>
+      <c r="AR18" s="40"/>
+      <c r="AS18" s="40"/>
+      <c r="AT18" s="40"/>
+      <c r="AU18" s="40"/>
+      <c r="AV18" s="40"/>
+      <c r="AW18" s="40"/>
+      <c r="AX18" s="40"/>
+      <c r="AY18" s="40"/>
+      <c r="AZ18" s="40"/>
+      <c r="BA18" s="40"/>
+      <c r="BB18" s="40"/>
+      <c r="BC18" s="40"/>
+      <c r="BD18" s="40"/>
+      <c r="BE18" s="40"/>
+      <c r="BF18" s="40"/>
+      <c r="BG18" s="40"/>
+      <c r="BH18" s="40"/>
+      <c r="BI18" s="40"/>
+      <c r="BJ18" s="40"/>
+      <c r="BK18" s="40"/>
     </row>
     <row r="19" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="B19" s="41" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C19" s="42">
         <v>0</v>
       </c>
       <c r="D19" s="81">
-        <v>46374</v>
+        <v>46348</v>
       </c>
       <c r="E19" s="81">
-        <v>46416</v>
+        <v>46355</v>
       </c>
       <c r="F19" s="13"/>
-      <c r="G19" s="4">
-        <f t="shared" si="5"/>
-        <v>43</v>
-      </c>
+      <c r="G19" s="4"/>
       <c r="H19" s="40"/>
       <c r="I19" s="40"/>
       <c r="J19" s="40"/>
@@ -3299,261 +3290,258 @@
     </row>
     <row r="20" spans="1:63" s="89" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="82"/>
-      <c r="B20" s="91" t="s">
-        <v>53</v>
-      </c>
-      <c r="C20" s="92">
-        <v>0.05</v>
-      </c>
-      <c r="D20" s="93">
-        <v>46508</v>
-      </c>
-      <c r="E20" s="93">
-        <v>46508</v>
+      <c r="B20" s="83" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="84">
+        <v>0</v>
+      </c>
+      <c r="D20" s="85">
+        <v>46371</v>
+      </c>
+      <c r="E20" s="85">
+        <v>46374</v>
       </c>
       <c r="F20" s="86"/>
       <c r="G20" s="87"/>
-      <c r="H20" s="94"/>
-      <c r="I20" s="94"/>
-      <c r="J20" s="94"/>
-      <c r="K20" s="94"/>
-      <c r="L20" s="94"/>
-      <c r="M20" s="94"/>
-      <c r="N20" s="94"/>
-      <c r="O20" s="94"/>
-      <c r="P20" s="94"/>
-      <c r="Q20" s="94"/>
-      <c r="R20" s="94"/>
-      <c r="S20" s="94"/>
-      <c r="T20" s="94"/>
-      <c r="U20" s="94"/>
-      <c r="V20" s="94"/>
-      <c r="W20" s="94"/>
-      <c r="X20" s="95"/>
-      <c r="Y20" s="94"/>
-      <c r="Z20" s="94"/>
-      <c r="AA20" s="94"/>
-      <c r="AB20" s="94"/>
-      <c r="AC20" s="94"/>
-      <c r="AD20" s="94"/>
-      <c r="AE20" s="94"/>
-      <c r="AF20" s="94"/>
-      <c r="AG20" s="94"/>
-      <c r="AH20" s="94"/>
-      <c r="AI20" s="94"/>
-      <c r="AJ20" s="94"/>
-      <c r="AK20" s="94"/>
-      <c r="AL20" s="94"/>
-      <c r="AM20" s="94"/>
-      <c r="AN20" s="94"/>
-      <c r="AO20" s="94"/>
-      <c r="AP20" s="94"/>
-      <c r="AQ20" s="94"/>
-      <c r="AR20" s="94"/>
-      <c r="AS20" s="94"/>
-      <c r="AT20" s="94"/>
-      <c r="AU20" s="94"/>
-      <c r="AV20" s="94"/>
-      <c r="AW20" s="94"/>
-      <c r="AX20" s="94"/>
-      <c r="AY20" s="94"/>
-      <c r="AZ20" s="94"/>
-      <c r="BA20" s="94"/>
-      <c r="BB20" s="94"/>
-      <c r="BC20" s="94"/>
-      <c r="BD20" s="94"/>
-      <c r="BE20" s="94"/>
-      <c r="BF20" s="94"/>
-      <c r="BG20" s="94"/>
-      <c r="BH20" s="94"/>
-      <c r="BI20" s="94"/>
-      <c r="BJ20" s="94"/>
-      <c r="BK20" s="94"/>
+      <c r="H20" s="88"/>
+      <c r="I20" s="88"/>
+      <c r="J20" s="88"/>
+      <c r="K20" s="88"/>
+      <c r="L20" s="88"/>
+      <c r="M20" s="88"/>
+      <c r="N20" s="88"/>
+      <c r="O20" s="88"/>
+      <c r="P20" s="88"/>
+      <c r="Q20" s="88"/>
+      <c r="R20" s="88"/>
+      <c r="S20" s="88"/>
+      <c r="T20" s="88"/>
+      <c r="U20" s="88"/>
+      <c r="V20" s="88"/>
+      <c r="W20" s="88"/>
+      <c r="X20" s="90"/>
+      <c r="Y20" s="88"/>
+      <c r="Z20" s="88"/>
+      <c r="AA20" s="88"/>
+      <c r="AB20" s="88"/>
+      <c r="AC20" s="88"/>
+      <c r="AD20" s="88"/>
+      <c r="AE20" s="88"/>
+      <c r="AF20" s="88"/>
+      <c r="AG20" s="88"/>
+      <c r="AH20" s="88"/>
+      <c r="AI20" s="88"/>
+      <c r="AJ20" s="88"/>
+      <c r="AK20" s="88"/>
+      <c r="AL20" s="88"/>
+      <c r="AM20" s="88"/>
+      <c r="AN20" s="88"/>
+      <c r="AO20" s="88"/>
+      <c r="AP20" s="88"/>
+      <c r="AQ20" s="88"/>
+      <c r="AR20" s="88"/>
+      <c r="AS20" s="88"/>
+      <c r="AT20" s="88"/>
+      <c r="AU20" s="88"/>
+      <c r="AV20" s="88"/>
+      <c r="AW20" s="88"/>
+      <c r="AX20" s="88"/>
+      <c r="AY20" s="88"/>
+      <c r="AZ20" s="88"/>
+      <c r="BA20" s="88"/>
+      <c r="BB20" s="88"/>
+      <c r="BC20" s="88"/>
+      <c r="BD20" s="88"/>
+      <c r="BE20" s="88"/>
+      <c r="BF20" s="88"/>
+      <c r="BG20" s="88"/>
+      <c r="BH20" s="88"/>
+      <c r="BI20" s="88"/>
+      <c r="BJ20" s="88"/>
+      <c r="BK20" s="88"/>
     </row>
     <row r="21" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="72"/>
-      <c r="B21" s="44" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="45"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="47"/>
+      <c r="A21" s="11"/>
+      <c r="B21" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="42">
+        <v>0</v>
+      </c>
+      <c r="D21" s="81">
+        <v>46374</v>
+      </c>
+      <c r="E21" s="81">
+        <v>46416</v>
+      </c>
       <c r="F21" s="13"/>
-      <c r="G21" s="4" t="str">
+      <c r="G21" s="4">
+        <f t="shared" si="5"/>
+        <v>43</v>
+      </c>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="40"/>
+      <c r="M21" s="40"/>
+      <c r="N21" s="40"/>
+      <c r="O21" s="40"/>
+      <c r="P21" s="40"/>
+      <c r="Q21" s="40"/>
+      <c r="R21" s="40"/>
+      <c r="S21" s="40"/>
+      <c r="T21" s="40"/>
+      <c r="U21" s="40"/>
+      <c r="V21" s="40"/>
+      <c r="W21" s="40"/>
+      <c r="X21" s="43"/>
+      <c r="Y21" s="40"/>
+      <c r="Z21" s="40"/>
+      <c r="AA21" s="40"/>
+      <c r="AB21" s="40"/>
+      <c r="AC21" s="40"/>
+      <c r="AD21" s="40"/>
+      <c r="AE21" s="40"/>
+      <c r="AF21" s="40"/>
+      <c r="AG21" s="40"/>
+      <c r="AH21" s="40"/>
+      <c r="AI21" s="40"/>
+      <c r="AJ21" s="40"/>
+      <c r="AK21" s="40"/>
+      <c r="AL21" s="40"/>
+      <c r="AM21" s="40"/>
+      <c r="AN21" s="40"/>
+      <c r="AO21" s="40"/>
+      <c r="AP21" s="40"/>
+      <c r="AQ21" s="40"/>
+      <c r="AR21" s="40"/>
+      <c r="AS21" s="40"/>
+      <c r="AT21" s="40"/>
+      <c r="AU21" s="40"/>
+      <c r="AV21" s="40"/>
+      <c r="AW21" s="40"/>
+      <c r="AX21" s="40"/>
+      <c r="AY21" s="40"/>
+      <c r="AZ21" s="40"/>
+      <c r="BA21" s="40"/>
+      <c r="BB21" s="40"/>
+      <c r="BC21" s="40"/>
+      <c r="BD21" s="40"/>
+      <c r="BE21" s="40"/>
+      <c r="BF21" s="40"/>
+      <c r="BG21" s="40"/>
+      <c r="BH21" s="40"/>
+      <c r="BI21" s="40"/>
+      <c r="BJ21" s="40"/>
+      <c r="BK21" s="40"/>
+    </row>
+    <row r="22" spans="1:63" s="89" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="82"/>
+      <c r="B22" s="91" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="92">
+        <v>0.05</v>
+      </c>
+      <c r="D22" s="93">
+        <v>46478</v>
+      </c>
+      <c r="E22" s="93">
+        <v>46508</v>
+      </c>
+      <c r="F22" s="86"/>
+      <c r="G22" s="87"/>
+      <c r="H22" s="94"/>
+      <c r="I22" s="94"/>
+      <c r="J22" s="94"/>
+      <c r="K22" s="94"/>
+      <c r="L22" s="94"/>
+      <c r="M22" s="94"/>
+      <c r="N22" s="94"/>
+      <c r="O22" s="94"/>
+      <c r="P22" s="94"/>
+      <c r="Q22" s="94"/>
+      <c r="R22" s="94"/>
+      <c r="S22" s="94"/>
+      <c r="T22" s="94"/>
+      <c r="U22" s="94"/>
+      <c r="V22" s="94"/>
+      <c r="W22" s="94"/>
+      <c r="X22" s="95"/>
+      <c r="Y22" s="94"/>
+      <c r="Z22" s="94"/>
+      <c r="AA22" s="94"/>
+      <c r="AB22" s="94"/>
+      <c r="AC22" s="94"/>
+      <c r="AD22" s="94"/>
+      <c r="AE22" s="94"/>
+      <c r="AF22" s="94"/>
+      <c r="AG22" s="94"/>
+      <c r="AH22" s="94"/>
+      <c r="AI22" s="94"/>
+      <c r="AJ22" s="94"/>
+      <c r="AK22" s="94"/>
+      <c r="AL22" s="94"/>
+      <c r="AM22" s="94"/>
+      <c r="AN22" s="94"/>
+      <c r="AO22" s="94"/>
+      <c r="AP22" s="94"/>
+      <c r="AQ22" s="94"/>
+      <c r="AR22" s="94"/>
+      <c r="AS22" s="94"/>
+      <c r="AT22" s="94"/>
+      <c r="AU22" s="94"/>
+      <c r="AV22" s="94"/>
+      <c r="AW22" s="94"/>
+      <c r="AX22" s="94"/>
+      <c r="AY22" s="94"/>
+      <c r="AZ22" s="94"/>
+      <c r="BA22" s="94"/>
+      <c r="BB22" s="94"/>
+      <c r="BC22" s="94"/>
+      <c r="BD22" s="94"/>
+      <c r="BE22" s="94"/>
+      <c r="BF22" s="94"/>
+      <c r="BG22" s="94"/>
+      <c r="BH22" s="94"/>
+      <c r="BI22" s="94"/>
+      <c r="BJ22" s="94"/>
+      <c r="BK22" s="94"/>
+    </row>
+    <row r="23" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="72"/>
+      <c r="B23" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="45"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="47"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="4" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="72"/>
-      <c r="B22" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="49">
-        <v>0.05</v>
-      </c>
-      <c r="D22" s="73">
-        <v>46309</v>
-      </c>
-      <c r="E22" s="73">
-        <v>46325</v>
-      </c>
-      <c r="F22" s="13"/>
-      <c r="G22" s="4">
-        <f t="shared" si="5"/>
-        <v>17</v>
-      </c>
-      <c r="H22" s="40"/>
-      <c r="I22" s="40"/>
-      <c r="J22" s="40"/>
-      <c r="K22" s="40"/>
-      <c r="L22" s="40"/>
-      <c r="M22" s="40"/>
-      <c r="N22" s="40"/>
-      <c r="O22" s="40"/>
-      <c r="P22" s="40"/>
-      <c r="Q22" s="40"/>
-      <c r="R22" s="40"/>
-      <c r="S22" s="40"/>
-      <c r="T22" s="40"/>
-      <c r="U22" s="40"/>
-      <c r="V22" s="40"/>
-      <c r="W22" s="40"/>
-      <c r="X22" s="40"/>
-      <c r="Y22" s="40"/>
-      <c r="Z22" s="40"/>
-      <c r="AA22" s="40"/>
-      <c r="AB22" s="40"/>
-      <c r="AC22" s="40"/>
-      <c r="AD22" s="40"/>
-      <c r="AE22" s="40"/>
-      <c r="AF22" s="40"/>
-      <c r="AG22" s="40"/>
-      <c r="AH22" s="40"/>
-      <c r="AI22" s="40"/>
-      <c r="AJ22" s="40"/>
-      <c r="AK22" s="40"/>
-      <c r="AL22" s="40"/>
-      <c r="AM22" s="40"/>
-      <c r="AN22" s="40"/>
-      <c r="AO22" s="40"/>
-      <c r="AP22" s="40"/>
-      <c r="AQ22" s="40"/>
-      <c r="AR22" s="40"/>
-      <c r="AS22" s="40"/>
-      <c r="AT22" s="40"/>
-      <c r="AU22" s="40"/>
-      <c r="AV22" s="40"/>
-      <c r="AW22" s="40"/>
-      <c r="AX22" s="40"/>
-      <c r="AY22" s="40"/>
-      <c r="AZ22" s="40"/>
-      <c r="BA22" s="40"/>
-      <c r="BB22" s="40"/>
-      <c r="BC22" s="40"/>
-      <c r="BD22" s="40"/>
-      <c r="BE22" s="40"/>
-      <c r="BF22" s="40"/>
-      <c r="BG22" s="40"/>
-      <c r="BH22" s="40"/>
-      <c r="BI22" s="40"/>
-      <c r="BJ22" s="40"/>
-      <c r="BK22" s="40"/>
-    </row>
-    <row r="23" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11"/>
-      <c r="B23" s="48" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="49">
-        <v>0.05</v>
-      </c>
-      <c r="D23" s="73">
-        <v>46317</v>
-      </c>
-      <c r="E23" s="73">
-        <v>46325</v>
-      </c>
-      <c r="F23" s="13"/>
-      <c r="G23" s="4">
-        <f t="shared" si="5"/>
-        <v>9</v>
-      </c>
-      <c r="H23" s="40"/>
-      <c r="I23" s="40"/>
-      <c r="J23" s="40"/>
-      <c r="K23" s="40"/>
-      <c r="L23" s="40"/>
-      <c r="M23" s="40"/>
-      <c r="N23" s="40"/>
-      <c r="O23" s="40"/>
-      <c r="P23" s="40"/>
-      <c r="Q23" s="40"/>
-      <c r="R23" s="40"/>
-      <c r="S23" s="40"/>
-      <c r="T23" s="43"/>
-      <c r="U23" s="43"/>
-      <c r="V23" s="40"/>
-      <c r="W23" s="40"/>
-      <c r="X23" s="40"/>
-      <c r="Y23" s="40"/>
-      <c r="Z23" s="40"/>
-      <c r="AA23" s="40"/>
-      <c r="AB23" s="40"/>
-      <c r="AC23" s="40"/>
-      <c r="AD23" s="40"/>
-      <c r="AE23" s="40"/>
-      <c r="AF23" s="40"/>
-      <c r="AG23" s="40"/>
-      <c r="AH23" s="40"/>
-      <c r="AI23" s="40"/>
-      <c r="AJ23" s="40"/>
-      <c r="AK23" s="40"/>
-      <c r="AL23" s="40"/>
-      <c r="AM23" s="40"/>
-      <c r="AN23" s="40"/>
-      <c r="AO23" s="40"/>
-      <c r="AP23" s="40"/>
-      <c r="AQ23" s="40"/>
-      <c r="AR23" s="40"/>
-      <c r="AS23" s="40"/>
-      <c r="AT23" s="40"/>
-      <c r="AU23" s="40"/>
-      <c r="AV23" s="40"/>
-      <c r="AW23" s="40"/>
-      <c r="AX23" s="40"/>
-      <c r="AY23" s="40"/>
-      <c r="AZ23" s="40"/>
-      <c r="BA23" s="40"/>
-      <c r="BB23" s="40"/>
-      <c r="BC23" s="40"/>
-      <c r="BD23" s="40"/>
-      <c r="BE23" s="40"/>
-      <c r="BF23" s="40"/>
-      <c r="BG23" s="40"/>
-      <c r="BH23" s="40"/>
-      <c r="BI23" s="40"/>
-      <c r="BJ23" s="40"/>
-      <c r="BK23" s="40"/>
-    </row>
     <row r="24" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11"/>
+      <c r="A24" s="72"/>
       <c r="B24" s="48" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="C24" s="49">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="D24" s="73">
-        <v>46327</v>
+        <v>46302</v>
       </c>
       <c r="E24" s="73">
-        <v>46357</v>
+        <v>46313</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="4">
         <f t="shared" si="5"/>
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H24" s="40"/>
       <c r="I24" s="40"/>
@@ -3615,23 +3603,21 @@
     <row r="25" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="B25" s="48" t="s">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="C25" s="49">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D25" s="73">
-        <f>D24</f>
-        <v>46327</v>
+        <v>46309</v>
       </c>
       <c r="E25" s="73">
-        <f>D25+2</f>
-        <v>46329</v>
+        <v>46325</v>
       </c>
       <c r="F25" s="13"/>
       <c r="G25" s="4">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="H25" s="40"/>
       <c r="I25" s="40"/>
@@ -3645,11 +3631,11 @@
       <c r="Q25" s="40"/>
       <c r="R25" s="40"/>
       <c r="S25" s="40"/>
-      <c r="T25" s="40"/>
-      <c r="U25" s="40"/>
+      <c r="T25" s="43"/>
+      <c r="U25" s="43"/>
       <c r="V25" s="40"/>
       <c r="W25" s="40"/>
-      <c r="X25" s="43"/>
+      <c r="X25" s="40"/>
       <c r="Y25" s="40"/>
       <c r="Z25" s="40"/>
       <c r="AA25" s="40"/>
@@ -3693,24 +3679,19 @@
     <row r="26" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11"/>
       <c r="B26" s="48" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="C26" s="49">
         <v>0</v>
       </c>
       <c r="D26" s="73">
-        <f>D25</f>
-        <v>46327</v>
+        <v>46313</v>
       </c>
       <c r="E26" s="73">
-        <f>D26+3</f>
-        <v>46330</v>
+        <v>46356</v>
       </c>
       <c r="F26" s="13"/>
-      <c r="G26" s="4">
-        <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
+      <c r="G26" s="4"/>
       <c r="H26" s="40"/>
       <c r="I26" s="40"/>
       <c r="J26" s="40"/>
@@ -3723,8 +3704,8 @@
       <c r="Q26" s="40"/>
       <c r="R26" s="40"/>
       <c r="S26" s="40"/>
-      <c r="T26" s="40"/>
-      <c r="U26" s="40"/>
+      <c r="T26" s="43"/>
+      <c r="U26" s="43"/>
       <c r="V26" s="40"/>
       <c r="W26" s="40"/>
       <c r="X26" s="40"/>
@@ -3770,170 +3751,168 @@
     </row>
     <row r="27" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11"/>
-      <c r="B27" s="50" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" s="51"/>
-      <c r="D27" s="74"/>
-      <c r="E27" s="75"/>
+      <c r="B27" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="49">
+        <v>0</v>
+      </c>
+      <c r="D27" s="73">
+        <v>46357</v>
+      </c>
+      <c r="E27" s="73">
+        <v>46363</v>
+      </c>
       <c r="F27" s="13"/>
-      <c r="G27" s="4" t="str">
+      <c r="G27" s="4">
+        <f t="shared" si="5"/>
+        <v>7</v>
+      </c>
+      <c r="H27" s="40"/>
+      <c r="I27" s="40"/>
+      <c r="J27" s="40"/>
+      <c r="K27" s="40"/>
+      <c r="L27" s="40"/>
+      <c r="M27" s="40"/>
+      <c r="N27" s="40"/>
+      <c r="O27" s="40"/>
+      <c r="P27" s="40"/>
+      <c r="Q27" s="40"/>
+      <c r="R27" s="40"/>
+      <c r="S27" s="40"/>
+      <c r="T27" s="40"/>
+      <c r="U27" s="40"/>
+      <c r="V27" s="40"/>
+      <c r="W27" s="40"/>
+      <c r="X27" s="40"/>
+      <c r="Y27" s="40"/>
+      <c r="Z27" s="40"/>
+      <c r="AA27" s="40"/>
+      <c r="AB27" s="40"/>
+      <c r="AC27" s="40"/>
+      <c r="AD27" s="40"/>
+      <c r="AE27" s="40"/>
+      <c r="AF27" s="40"/>
+      <c r="AG27" s="40"/>
+      <c r="AH27" s="40"/>
+      <c r="AI27" s="40"/>
+      <c r="AJ27" s="40"/>
+      <c r="AK27" s="40"/>
+      <c r="AL27" s="40"/>
+      <c r="AM27" s="40"/>
+      <c r="AN27" s="40"/>
+      <c r="AO27" s="40"/>
+      <c r="AP27" s="40"/>
+      <c r="AQ27" s="40"/>
+      <c r="AR27" s="40"/>
+      <c r="AS27" s="40"/>
+      <c r="AT27" s="40"/>
+      <c r="AU27" s="40"/>
+      <c r="AV27" s="40"/>
+      <c r="AW27" s="40"/>
+      <c r="AX27" s="40"/>
+      <c r="AY27" s="40"/>
+      <c r="AZ27" s="40"/>
+      <c r="BA27" s="40"/>
+      <c r="BB27" s="40"/>
+      <c r="BC27" s="40"/>
+      <c r="BD27" s="40"/>
+      <c r="BE27" s="40"/>
+      <c r="BF27" s="40"/>
+      <c r="BG27" s="40"/>
+      <c r="BH27" s="40"/>
+      <c r="BI27" s="40"/>
+      <c r="BJ27" s="40"/>
+      <c r="BK27" s="40"/>
+    </row>
+    <row r="28" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="11"/>
+      <c r="B28" s="50" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="51"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="75"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="4" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="H27" s="52"/>
-      <c r="I27" s="52"/>
-      <c r="J27" s="52"/>
-      <c r="K27" s="52"/>
-      <c r="L27" s="52"/>
-      <c r="M27" s="52"/>
-      <c r="N27" s="52"/>
-      <c r="O27" s="52"/>
-      <c r="P27" s="52"/>
-      <c r="Q27" s="52"/>
-      <c r="R27" s="52"/>
-      <c r="S27" s="52"/>
-      <c r="T27" s="52"/>
-      <c r="U27" s="52"/>
-      <c r="V27" s="52"/>
-      <c r="W27" s="52"/>
-      <c r="X27" s="52"/>
-      <c r="Y27" s="52"/>
-      <c r="Z27" s="52"/>
-      <c r="AA27" s="52"/>
-      <c r="AB27" s="52"/>
-      <c r="AC27" s="52"/>
-      <c r="AD27" s="52"/>
-      <c r="AE27" s="52"/>
-      <c r="AF27" s="52"/>
-      <c r="AG27" s="52"/>
-      <c r="AH27" s="52"/>
-      <c r="AI27" s="52"/>
-      <c r="AJ27" s="52"/>
-      <c r="AK27" s="52"/>
-      <c r="AL27" s="52"/>
-      <c r="AM27" s="52"/>
-      <c r="AN27" s="52"/>
-      <c r="AO27" s="52"/>
-      <c r="AP27" s="52"/>
-      <c r="AQ27" s="52"/>
-      <c r="AR27" s="52"/>
-      <c r="AS27" s="52"/>
-      <c r="AT27" s="52"/>
-      <c r="AU27" s="52"/>
-      <c r="AV27" s="52"/>
-      <c r="AW27" s="52"/>
-      <c r="AX27" s="52"/>
-      <c r="AY27" s="52"/>
-      <c r="AZ27" s="52"/>
-      <c r="BA27" s="52"/>
-      <c r="BB27" s="52"/>
-      <c r="BC27" s="52"/>
-      <c r="BD27" s="52"/>
-      <c r="BE27" s="52"/>
-      <c r="BF27" s="52"/>
-      <c r="BG27" s="52"/>
-      <c r="BH27" s="52"/>
-      <c r="BI27" s="52"/>
-      <c r="BJ27" s="52"/>
-      <c r="BK27" s="52"/>
-    </row>
-    <row r="28" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11"/>
-      <c r="B28" s="53" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" s="54">
-        <v>0</v>
-      </c>
-      <c r="D28" s="76">
-        <f>D9+15</f>
-        <v>46301</v>
-      </c>
-      <c r="E28" s="76">
-        <f>D28+5</f>
-        <v>46306</v>
-      </c>
-      <c r="F28" s="13"/>
-      <c r="G28" s="4">
-        <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="H28" s="40"/>
-      <c r="I28" s="40"/>
-      <c r="J28" s="40"/>
-      <c r="K28" s="40"/>
-      <c r="L28" s="40"/>
-      <c r="M28" s="40"/>
-      <c r="N28" s="40"/>
-      <c r="O28" s="40"/>
-      <c r="P28" s="40"/>
-      <c r="Q28" s="40"/>
-      <c r="R28" s="40"/>
-      <c r="S28" s="40"/>
-      <c r="T28" s="40"/>
-      <c r="U28" s="40"/>
-      <c r="V28" s="40"/>
-      <c r="W28" s="40"/>
-      <c r="X28" s="40"/>
-      <c r="Y28" s="40"/>
-      <c r="Z28" s="40"/>
-      <c r="AA28" s="40"/>
-      <c r="AB28" s="40"/>
-      <c r="AC28" s="40"/>
-      <c r="AD28" s="40"/>
-      <c r="AE28" s="40"/>
-      <c r="AF28" s="40"/>
-      <c r="AG28" s="40"/>
-      <c r="AH28" s="40"/>
-      <c r="AI28" s="40"/>
-      <c r="AJ28" s="40"/>
-      <c r="AK28" s="40"/>
-      <c r="AL28" s="40"/>
-      <c r="AM28" s="40"/>
-      <c r="AN28" s="40"/>
-      <c r="AO28" s="40"/>
-      <c r="AP28" s="40"/>
-      <c r="AQ28" s="40"/>
-      <c r="AR28" s="40"/>
-      <c r="AS28" s="40"/>
-      <c r="AT28" s="40"/>
-      <c r="AU28" s="40"/>
-      <c r="AV28" s="40"/>
-      <c r="AW28" s="40"/>
-      <c r="AX28" s="40"/>
-      <c r="AY28" s="40"/>
-      <c r="AZ28" s="40"/>
-      <c r="BA28" s="40"/>
-      <c r="BB28" s="40"/>
-      <c r="BC28" s="40"/>
-      <c r="BD28" s="40"/>
-      <c r="BE28" s="40"/>
-      <c r="BF28" s="40"/>
-      <c r="BG28" s="40"/>
-      <c r="BH28" s="40"/>
-      <c r="BI28" s="40"/>
-      <c r="BJ28" s="40"/>
-      <c r="BK28" s="40"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="52"/>
+      <c r="J28" s="52"/>
+      <c r="K28" s="52"/>
+      <c r="L28" s="52"/>
+      <c r="M28" s="52"/>
+      <c r="N28" s="52"/>
+      <c r="O28" s="52"/>
+      <c r="P28" s="52"/>
+      <c r="Q28" s="52"/>
+      <c r="R28" s="52"/>
+      <c r="S28" s="52"/>
+      <c r="T28" s="52"/>
+      <c r="U28" s="52"/>
+      <c r="V28" s="52"/>
+      <c r="W28" s="52"/>
+      <c r="X28" s="52"/>
+      <c r="Y28" s="52"/>
+      <c r="Z28" s="52"/>
+      <c r="AA28" s="52"/>
+      <c r="AB28" s="52"/>
+      <c r="AC28" s="52"/>
+      <c r="AD28" s="52"/>
+      <c r="AE28" s="52"/>
+      <c r="AF28" s="52"/>
+      <c r="AG28" s="52"/>
+      <c r="AH28" s="52"/>
+      <c r="AI28" s="52"/>
+      <c r="AJ28" s="52"/>
+      <c r="AK28" s="52"/>
+      <c r="AL28" s="52"/>
+      <c r="AM28" s="52"/>
+      <c r="AN28" s="52"/>
+      <c r="AO28" s="52"/>
+      <c r="AP28" s="52"/>
+      <c r="AQ28" s="52"/>
+      <c r="AR28" s="52"/>
+      <c r="AS28" s="52"/>
+      <c r="AT28" s="52"/>
+      <c r="AU28" s="52"/>
+      <c r="AV28" s="52"/>
+      <c r="AW28" s="52"/>
+      <c r="AX28" s="52"/>
+      <c r="AY28" s="52"/>
+      <c r="AZ28" s="52"/>
+      <c r="BA28" s="52"/>
+      <c r="BB28" s="52"/>
+      <c r="BC28" s="52"/>
+      <c r="BD28" s="52"/>
+      <c r="BE28" s="52"/>
+      <c r="BF28" s="52"/>
+      <c r="BG28" s="52"/>
+      <c r="BH28" s="52"/>
+      <c r="BI28" s="52"/>
+      <c r="BJ28" s="52"/>
+      <c r="BK28" s="52"/>
     </row>
     <row r="29" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11"/>
       <c r="B29" s="53" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C29" s="54">
         <v>0</v>
       </c>
       <c r="D29" s="76">
-        <v>46419</v>
+        <v>46357</v>
       </c>
       <c r="E29" s="76">
-        <v>46447</v>
+        <v>46374</v>
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="4">
         <f t="shared" si="5"/>
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="H29" s="40"/>
       <c r="I29" s="40"/>
@@ -3995,21 +3974,21 @@
     <row r="30" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11"/>
       <c r="B30" s="53" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="C30" s="54">
         <v>0</v>
       </c>
       <c r="D30" s="76">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="E30" s="76">
-        <v>46456</v>
+        <v>46439</v>
       </c>
       <c r="F30" s="13"/>
       <c r="G30" s="4">
         <f t="shared" si="5"/>
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="H30" s="40"/>
       <c r="I30" s="40"/>
@@ -4071,23 +4050,21 @@
     <row r="31" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11"/>
       <c r="B31" s="53" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="C31" s="54">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D31" s="76">
-        <f>E30+1</f>
-        <v>46457</v>
+        <v>46439</v>
       </c>
       <c r="E31" s="76">
-        <f>D31+4</f>
-        <v>46461</v>
+        <v>46447</v>
       </c>
       <c r="F31" s="13"/>
       <c r="G31" s="4">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H31" s="40"/>
       <c r="I31" s="40"/>
@@ -4149,23 +4126,21 @@
     <row r="32" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11"/>
       <c r="B32" s="53" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="C32" s="54">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D32" s="76">
-        <f>D30</f>
         <v>46447</v>
       </c>
       <c r="E32" s="76">
-        <f>D32+4</f>
-        <v>46451</v>
+        <v>46453</v>
       </c>
       <c r="F32" s="13"/>
       <c r="G32" s="4">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H32" s="40"/>
       <c r="I32" s="40"/>
@@ -4226,172 +4201,168 @@
     </row>
     <row r="33" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11"/>
-      <c r="B33" s="55" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" s="56"/>
-      <c r="D33" s="77"/>
-      <c r="E33" s="78"/>
+      <c r="B33" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" s="54">
+        <v>0</v>
+      </c>
+      <c r="D33" s="76">
+        <v>46453</v>
+      </c>
+      <c r="E33" s="76">
+        <v>46460</v>
+      </c>
       <c r="F33" s="13"/>
-      <c r="G33" s="4" t="str">
+      <c r="G33" s="4">
+        <f t="shared" si="5"/>
+        <v>8</v>
+      </c>
+      <c r="H33" s="40"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="40"/>
+      <c r="M33" s="40"/>
+      <c r="N33" s="40"/>
+      <c r="O33" s="40"/>
+      <c r="P33" s="40"/>
+      <c r="Q33" s="40"/>
+      <c r="R33" s="40"/>
+      <c r="S33" s="40"/>
+      <c r="T33" s="40"/>
+      <c r="U33" s="40"/>
+      <c r="V33" s="40"/>
+      <c r="W33" s="40"/>
+      <c r="X33" s="40"/>
+      <c r="Y33" s="40"/>
+      <c r="Z33" s="40"/>
+      <c r="AA33" s="40"/>
+      <c r="AB33" s="40"/>
+      <c r="AC33" s="40"/>
+      <c r="AD33" s="40"/>
+      <c r="AE33" s="40"/>
+      <c r="AF33" s="40"/>
+      <c r="AG33" s="40"/>
+      <c r="AH33" s="40"/>
+      <c r="AI33" s="40"/>
+      <c r="AJ33" s="40"/>
+      <c r="AK33" s="40"/>
+      <c r="AL33" s="40"/>
+      <c r="AM33" s="40"/>
+      <c r="AN33" s="40"/>
+      <c r="AO33" s="40"/>
+      <c r="AP33" s="40"/>
+      <c r="AQ33" s="40"/>
+      <c r="AR33" s="40"/>
+      <c r="AS33" s="40"/>
+      <c r="AT33" s="40"/>
+      <c r="AU33" s="40"/>
+      <c r="AV33" s="40"/>
+      <c r="AW33" s="40"/>
+      <c r="AX33" s="40"/>
+      <c r="AY33" s="40"/>
+      <c r="AZ33" s="40"/>
+      <c r="BA33" s="40"/>
+      <c r="BB33" s="40"/>
+      <c r="BC33" s="40"/>
+      <c r="BD33" s="40"/>
+      <c r="BE33" s="40"/>
+      <c r="BF33" s="40"/>
+      <c r="BG33" s="40"/>
+      <c r="BH33" s="40"/>
+      <c r="BI33" s="40"/>
+      <c r="BJ33" s="40"/>
+      <c r="BK33" s="40"/>
+    </row>
+    <row r="34" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="11"/>
+      <c r="B34" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="56"/>
+      <c r="D34" s="77"/>
+      <c r="E34" s="78"/>
+      <c r="F34" s="13"/>
+      <c r="G34" s="4" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="H33" s="57"/>
-      <c r="I33" s="57"/>
-      <c r="J33" s="57"/>
-      <c r="K33" s="57"/>
-      <c r="L33" s="57"/>
-      <c r="M33" s="57"/>
-      <c r="N33" s="57"/>
-      <c r="O33" s="57"/>
-      <c r="P33" s="57"/>
-      <c r="Q33" s="57"/>
-      <c r="R33" s="57"/>
-      <c r="S33" s="57"/>
-      <c r="T33" s="57"/>
-      <c r="U33" s="57"/>
-      <c r="V33" s="57"/>
-      <c r="W33" s="57"/>
-      <c r="X33" s="57"/>
-      <c r="Y33" s="57"/>
-      <c r="Z33" s="57"/>
-      <c r="AA33" s="57"/>
-      <c r="AB33" s="57"/>
-      <c r="AC33" s="57"/>
-      <c r="AD33" s="57"/>
-      <c r="AE33" s="57"/>
-      <c r="AF33" s="57"/>
-      <c r="AG33" s="57"/>
-      <c r="AH33" s="57"/>
-      <c r="AI33" s="57"/>
-      <c r="AJ33" s="57"/>
-      <c r="AK33" s="57"/>
-      <c r="AL33" s="57"/>
-      <c r="AM33" s="57"/>
-      <c r="AN33" s="57"/>
-      <c r="AO33" s="57"/>
-      <c r="AP33" s="57"/>
-      <c r="AQ33" s="57"/>
-      <c r="AR33" s="57"/>
-      <c r="AS33" s="57"/>
-      <c r="AT33" s="57"/>
-      <c r="AU33" s="57"/>
-      <c r="AV33" s="57"/>
-      <c r="AW33" s="57"/>
-      <c r="AX33" s="57"/>
-      <c r="AY33" s="57"/>
-      <c r="AZ33" s="57"/>
-      <c r="BA33" s="57"/>
-      <c r="BB33" s="57"/>
-      <c r="BC33" s="57"/>
-      <c r="BD33" s="57"/>
-      <c r="BE33" s="57"/>
-      <c r="BF33" s="57"/>
-      <c r="BG33" s="57"/>
-      <c r="BH33" s="57"/>
-      <c r="BI33" s="57"/>
-      <c r="BJ33" s="57"/>
-      <c r="BK33" s="57"/>
-    </row>
-    <row r="34" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="11"/>
-      <c r="B34" s="58" t="s">
-        <v>10</v>
-      </c>
-      <c r="C34" s="59">
-        <v>0.25</v>
-      </c>
-      <c r="D34" s="79">
-        <f>D28+2</f>
-        <v>46303</v>
-      </c>
-      <c r="E34" s="79">
-        <f>D34+3</f>
-        <v>46306</v>
-      </c>
-      <c r="F34" s="13"/>
-      <c r="G34" s="4">
-        <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="H34" s="40"/>
-      <c r="I34" s="40"/>
-      <c r="J34" s="40"/>
-      <c r="K34" s="40"/>
-      <c r="L34" s="40"/>
-      <c r="M34" s="40"/>
-      <c r="N34" s="40"/>
-      <c r="O34" s="40"/>
-      <c r="P34" s="40"/>
-      <c r="Q34" s="40"/>
-      <c r="R34" s="40"/>
-      <c r="S34" s="40"/>
-      <c r="T34" s="40"/>
-      <c r="U34" s="40"/>
-      <c r="V34" s="40"/>
-      <c r="W34" s="40"/>
-      <c r="X34" s="40"/>
-      <c r="Y34" s="40"/>
-      <c r="Z34" s="40"/>
-      <c r="AA34" s="40"/>
-      <c r="AB34" s="40"/>
-      <c r="AC34" s="40"/>
-      <c r="AD34" s="40"/>
-      <c r="AE34" s="40"/>
-      <c r="AF34" s="40"/>
-      <c r="AG34" s="40"/>
-      <c r="AH34" s="40"/>
-      <c r="AI34" s="40"/>
-      <c r="AJ34" s="40"/>
-      <c r="AK34" s="40"/>
-      <c r="AL34" s="40"/>
-      <c r="AM34" s="40"/>
-      <c r="AN34" s="40"/>
-      <c r="AO34" s="40"/>
-      <c r="AP34" s="40"/>
-      <c r="AQ34" s="40"/>
-      <c r="AR34" s="40"/>
-      <c r="AS34" s="40"/>
-      <c r="AT34" s="40"/>
-      <c r="AU34" s="40"/>
-      <c r="AV34" s="40"/>
-      <c r="AW34" s="40"/>
-      <c r="AX34" s="40"/>
-      <c r="AY34" s="40"/>
-      <c r="AZ34" s="40"/>
-      <c r="BA34" s="40"/>
-      <c r="BB34" s="40"/>
-      <c r="BC34" s="40"/>
-      <c r="BD34" s="40"/>
-      <c r="BE34" s="40"/>
-      <c r="BF34" s="40"/>
-      <c r="BG34" s="40"/>
-      <c r="BH34" s="40"/>
-      <c r="BI34" s="40"/>
-      <c r="BJ34" s="40"/>
-      <c r="BK34" s="40"/>
+      <c r="H34" s="57"/>
+      <c r="I34" s="57"/>
+      <c r="J34" s="57"/>
+      <c r="K34" s="57"/>
+      <c r="L34" s="57"/>
+      <c r="M34" s="57"/>
+      <c r="N34" s="57"/>
+      <c r="O34" s="57"/>
+      <c r="P34" s="57"/>
+      <c r="Q34" s="57"/>
+      <c r="R34" s="57"/>
+      <c r="S34" s="57"/>
+      <c r="T34" s="57"/>
+      <c r="U34" s="57"/>
+      <c r="V34" s="57"/>
+      <c r="W34" s="57"/>
+      <c r="X34" s="57"/>
+      <c r="Y34" s="57"/>
+      <c r="Z34" s="57"/>
+      <c r="AA34" s="57"/>
+      <c r="AB34" s="57"/>
+      <c r="AC34" s="57"/>
+      <c r="AD34" s="57"/>
+      <c r="AE34" s="57"/>
+      <c r="AF34" s="57"/>
+      <c r="AG34" s="57"/>
+      <c r="AH34" s="57"/>
+      <c r="AI34" s="57"/>
+      <c r="AJ34" s="57"/>
+      <c r="AK34" s="57"/>
+      <c r="AL34" s="57"/>
+      <c r="AM34" s="57"/>
+      <c r="AN34" s="57"/>
+      <c r="AO34" s="57"/>
+      <c r="AP34" s="57"/>
+      <c r="AQ34" s="57"/>
+      <c r="AR34" s="57"/>
+      <c r="AS34" s="57"/>
+      <c r="AT34" s="57"/>
+      <c r="AU34" s="57"/>
+      <c r="AV34" s="57"/>
+      <c r="AW34" s="57"/>
+      <c r="AX34" s="57"/>
+      <c r="AY34" s="57"/>
+      <c r="AZ34" s="57"/>
+      <c r="BA34" s="57"/>
+      <c r="BB34" s="57"/>
+      <c r="BC34" s="57"/>
+      <c r="BD34" s="57"/>
+      <c r="BE34" s="57"/>
+      <c r="BF34" s="57"/>
+      <c r="BG34" s="57"/>
+      <c r="BH34" s="57"/>
+      <c r="BI34" s="57"/>
+      <c r="BJ34" s="57"/>
+      <c r="BK34" s="57"/>
     </row>
     <row r="35" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11"/>
       <c r="B35" s="58" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C35" s="59">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D35" s="79">
-        <f>E34</f>
-        <v>46306</v>
+        <v>46340</v>
       </c>
       <c r="E35" s="79">
-        <f>D35+4</f>
-        <v>46310</v>
+        <v>46374</v>
       </c>
       <c r="F35" s="13"/>
       <c r="G35" s="4">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="H35" s="40"/>
       <c r="I35" s="40"/>
@@ -4453,23 +4424,21 @@
     <row r="36" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11"/>
       <c r="B36" s="58" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="C36" s="59">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D36" s="79">
-        <f>E35+1</f>
-        <v>46311</v>
+        <v>46439</v>
       </c>
       <c r="E36" s="79">
-        <f>D36+3</f>
-        <v>46314</v>
+        <v>46447</v>
       </c>
       <c r="F36" s="13"/>
       <c r="G36" s="4">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H36" s="40"/>
       <c r="I36" s="40"/>
@@ -4531,18 +4500,18 @@
     <row r="37" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11"/>
       <c r="B37" s="58" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="C37" s="59">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D37" s="79">
-        <f>D34+5</f>
-        <v>46308</v>
+        <f>E36+1</f>
+        <v>46448</v>
       </c>
       <c r="E37" s="79">
         <f>D37+3</f>
-        <v>46311</v>
+        <v>46451</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="4">
@@ -4609,23 +4578,21 @@
     <row r="38" spans="1:63" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11"/>
       <c r="B38" s="58" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="C38" s="59">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D38" s="79">
-        <f>D34+7</f>
-        <v>46310</v>
+        <v>46478</v>
       </c>
       <c r="E38" s="79">
-        <f>D38+5</f>
-        <v>46315</v>
+        <v>46508</v>
       </c>
       <c r="F38" s="13"/>
       <c r="G38" s="4">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="H38" s="40"/>
       <c r="I38" s="40"/>
@@ -4760,11 +4727,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="P2:Y2"/>
     <mergeCell ref="P1:Y1"/>
     <mergeCell ref="H1:N1"/>
@@ -4777,6 +4739,11 @@
     <mergeCell ref="AJ4:AP4"/>
     <mergeCell ref="AQ4:AW4"/>
     <mergeCell ref="AX4:BD4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C39">
     <cfRule type="dataBar" priority="23">
@@ -4797,7 +4764,7 @@
       <formula>AND(TODAY()&gt;=H$5, TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:BK20">
+  <conditionalFormatting sqref="H9:BK22">
     <cfRule type="expression" dxfId="7" priority="6">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -4805,7 +4772,7 @@
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H22:BK26">
+  <conditionalFormatting sqref="H24:BK27">
     <cfRule type="expression" dxfId="5" priority="4">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -4813,7 +4780,7 @@
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H28:BK32">
+  <conditionalFormatting sqref="H29:BK33">
     <cfRule type="expression" dxfId="3" priority="2">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -4821,7 +4788,7 @@
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H34:BK38">
+  <conditionalFormatting sqref="H35:BK38">
     <cfRule type="expression" dxfId="1" priority="36">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -4840,10 +4807,10 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Cells I5 through BL5 contain the day number for the week represented in the cell block above each date and are auto calculated._x000a__x000a_Today's date is outlined from today's date in row 5 through the entire date column to the end of the project schedule." sqref="A5:A6" xr:uid="{7A3789A6-A3FB-43B6-A4F7-8C0AC564F67E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Cell B8 contains the Phase 1 sample title. Enter a new title in cell B8._x000a_To delete the phase and work only from tasks, simply delete this row." sqref="A8" xr:uid="{CEC78982-AFA8-419E-B0A2-676B709E5100}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="B9 contains the task name.  C9 is the assignee.  D9 is a progress bar that shades based on the number entered into the cell.  _x000a__x000a_E9 contains the start date and F9 contains the end date._x000a__x000a_The Gantt chart will fill in starting in cell I9 based on task dates." sqref="A9" xr:uid="{D870A2F6-6B07-4F5A-A81D-4BCCFADF8796}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Rows 10 through 13 repeat the pattern from row 9. _x000a__x000a_Repeat the instructions from cell A9 for all task rows in this worksheet. _x000a__x000a_Continue entering tasks in cells A10 through A13 or go to cell A14 to learn more." sqref="A10:A12" xr:uid="{872449A7-C3CC-45B6-BA90-B1AAD66BA0E5}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Cell B14 contains the Phase 2 sample title. Enter a new title in cell B14._x000a_To delete the phase and work only from tasks, simply delete this row. To remove the phase, simply delete the row. Add tasks to previous phase by entering a new row above this one._x000a_" sqref="A21" xr:uid="{4F48FC41-E335-47F1-87AA-3333A52AD81C}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Phase 3's sample block starts in cell B20." sqref="A27" xr:uid="{956902D1-D3B5-416D-BB69-9362D193BC0A}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Phase 4's sample block starts in cell B26." sqref="A33" xr:uid="{DE54E5DE-526D-4D71-8D03-E99B4AB2FEE5}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Cell B14 contains the Phase 2 sample title. Enter a new title in cell B14._x000a_To delete the phase and work only from tasks, simply delete this row. To remove the phase, simply delete the row. Add tasks to previous phase by entering a new row above this one._x000a_" sqref="A23" xr:uid="{4F48FC41-E335-47F1-87AA-3333A52AD81C}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Phase 3's sample block starts in cell B20." sqref="A28" xr:uid="{956902D1-D3B5-416D-BB69-9362D193BC0A}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Phase 4's sample block starts in cell B26." sqref="A34" xr:uid="{DE54E5DE-526D-4D71-8D03-E99B4AB2FEE5}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Rows 10 through 13 repeat the pattern from row 9. _x000a__x000a_Repeat the instructions from cell A9 for all task rows in this worksheet. _x000a__x000a_Continue entering tasks in cells A10 through A13 or go to cell A14 to learn more." sqref="A10 A11:A14" xr:uid="{872449A7-C3CC-45B6-BA90-B1AAD66BA0E5}"/>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -4854,9 +4821,6 @@
   <headerFooter differentFirst="1" scaleWithDoc="0">
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
-  <ignoredErrors>
-    <ignoredError sqref="E25 E35" formula="1"/>
-  </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -4903,67 +4867,67 @@
     </row>
     <row r="4" spans="1:2" s="8" customFormat="1" ht="31.5" x14ac:dyDescent="0.6">
       <c r="A4" s="67" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="74.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="68" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="67" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="5" customFormat="1" ht="205.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="69" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="8" customFormat="1" ht="31.5" x14ac:dyDescent="0.6">
       <c r="A8" s="67" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="57" x14ac:dyDescent="0.2">
       <c r="A9" s="68" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="5" customFormat="1" ht="28.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="70" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="8" customFormat="1" ht="31.5" x14ac:dyDescent="0.6">
       <c r="A11" s="67" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A12" s="68" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="5" customFormat="1" ht="28.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="70" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="8" customFormat="1" ht="31.5" x14ac:dyDescent="0.6">
       <c r="A14" s="67" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="68" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A16" s="68" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
@@ -5003,23 +4967,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5335,22 +5288,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5377,9 +5337,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>